<commit_message>
Dados atualizados via Robô: 01/10/2026 16:15
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -914,7 +914,7 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="X3" s="4" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y3" s="4" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-movimentacoes-automaticas-curto-prazo/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-movimentacoes-automaticas-rf-simples/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-plus-mm-credito-privado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-rf-credito-privado-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -3589,12 +3589,12 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>09.548.729/0001-71</t>
+          <t>03.191.874/0001-61</t>
         </is>
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>5414</t>
+          <t>46</t>
         </is>
       </c>
       <c r="S13" s="4" t="inlineStr">
@@ -3604,27 +3604,27 @@
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
         <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
           <t>100.0</t>
         </is>
       </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
       <c r="W13" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="X13" s="4" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Y13" s="4" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
+          <t>IPCA+6%</t>
         </is>
       </c>
       <c r="AC13" s="4" t="inlineStr">
@@ -3694,12 +3694,12 @@
       </c>
       <c r="AL13" s="4" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM13" s="4" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN13" s="4" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="AR13" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FOCO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS13" s="4" t="inlineStr">
@@ -3730,43 +3730,43 @@
       </c>
       <c r="AT13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5414.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
         </is>
       </c>
       <c r="AU13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5414.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
         </is>
       </c>
       <c r="AV13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5414.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
         </is>
       </c>
       <c r="AW13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5414.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
         </is>
       </c>
       <c r="AX13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5414.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
       <c r="AY13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5414.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
         </is>
       </c>
       <c r="AZ13" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5414.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
         </is>
       </c>
       <c r="BA13" s="4" t="inlineStr"/>
       <c r="BB13" s="4" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/a5ab94de-1f04-4f00-87d2-ffa0c6babbaf?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-smart-infraestrutura-debincentivadas-cdi-rf-cred-priv-lp-subclasse-varejo/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>67.702.501/0001-90</t>
@@ -7466,15 +7470,19 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-vinland-debenture-incentivado/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>58.113.332/0001-62</t>
+          <t>10.646.888/0001-98</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>7931</t>
+          <t>5156</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
@@ -7484,7 +7492,7 @@
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr">
@@ -7514,22 +7522,22 @@
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
-          <t>D+13 (du)</t>
+          <t>D+0 (du)</t>
         </is>
       </c>
       <c r="AA28" s="2" t="inlineStr">
         <is>
-          <t>D+15 (du)</t>
+          <t>D+00 (du)</t>
         </is>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>RF Crédito Privado permite Risco Mercado</t>
+          <t>RF Crédito Privado sem Risco Mercado</t>
         </is>
       </c>
       <c r="AD28" s="2" t="inlineStr">
@@ -7549,33 +7557,37 @@
       </c>
       <c r="AG28" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="AH28" s="2" t="inlineStr">
         <is>
-          <t>13h00</t>
+          <t>17h00</t>
         </is>
       </c>
       <c r="AI28" s="2" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Sim · Automatico · 90%</t>
         </is>
       </c>
       <c r="AJ28" s="2" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="AK28" s="2" t="inlineStr"/>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK28" s="2" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
       <c r="AL28" s="2" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AM28" s="2" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AN28" s="2" t="inlineStr">
@@ -7596,43 +7608,47 @@
       </c>
       <c r="AR28" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT SULAMÉRICA CRÉDITO ATIVO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PR</t>
-        </is>
-      </c>
-      <c r="AS28" s="2" t="inlineStr"/>
+          <t>CAIXA EXPERTISE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS28" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
       <c r="AT28" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7931.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5156.pdf</t>
         </is>
       </c>
       <c r="AU28" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7931.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5156.pdf</t>
         </is>
       </c>
       <c r="AV28" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7931.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5156.pdf</t>
         </is>
       </c>
       <c r="AW28" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7931.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5156.pdf</t>
         </is>
       </c>
       <c r="AX28" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7931.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5156.pdf</t>
         </is>
       </c>
       <c r="AY28" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7931.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5156.pdf</t>
         </is>
       </c>
       <c r="AZ28" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7931.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5156.pdf</t>
         </is>
       </c>
       <c r="BA28" s="2" t="inlineStr"/>
@@ -7714,7 +7730,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-arx-ipca-deb-incentivadas-rf-cred-priv-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>60.138.811/0001-85</t>
@@ -8986,7 +9006,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-rb-asset-deb-incentivadas-cdi-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>62.890.286/0001-85</t>
@@ -9236,7 +9260,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-unique-private-cred-priv-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-unique-private-cred-priv-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q35" s="4" t="inlineStr">
@@ -9496,7 +9520,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fif-inflacao-2027</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fif-inflacao-2027/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
@@ -10017,7 +10041,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-qualificado-rf-credito-privado-longo-prazo</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-qualificado-rf-credito-privado-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -10920,11 +10944,7 @@
           <t>CAIXA INDEXA TESOURO SELIC FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO – RESP LIMITADA</t>
         </is>
       </c>
-      <c r="AS41" s="4" t="inlineStr">
-        <is>
-          <t>OBS: Limite máximo por CPF - R$ 100.000,00</t>
-        </is>
-      </c>
+      <c r="AS41" s="4" t="inlineStr"/>
       <c r="AT41" s="4" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5940.pdf</t>
@@ -11041,7 +11061,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-renda-fixa-ativa-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-renda-fixa-ativa-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
@@ -11963,8 +11983,7 @@
       </c>
       <c r="AS45" s="4" t="inlineStr">
         <is>
-          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social). Há incidência de taxa de saída no Fundo, conforme exposto no Regulamento.
-Aberto para novas aplicações a partir de 01/12/2025, inclusive.</t>
+          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social). Há incidência de taxa de saída no Fundo, conforme exposto no Regulamento.</t>
         </is>
       </c>
       <c r="AT45" s="4" t="inlineStr">
@@ -12903,7 +12922,7 @@
       </c>
       <c r="X49" s="4" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y49" s="4" t="inlineStr">
@@ -13383,17 +13402,17 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/referenciados/fic-sigma-ref-di-longo-prazo</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-omega-private-ref-di-longo-prazo</t>
         </is>
       </c>
       <c r="Q51" s="4" t="inlineStr">
         <is>
-          <t>10.731.794/0001-17</t>
+          <t>55.036.101/0001-04</t>
         </is>
       </c>
       <c r="R51" s="4" t="inlineStr">
         <is>
-          <t>5171</t>
+          <t>7914</t>
         </is>
       </c>
       <c r="S51" s="4" t="inlineStr">
@@ -13403,12 +13422,12 @@
       </c>
       <c r="T51" s="4" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="U51" s="4" t="inlineStr">
         <is>
-          <t>50000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V51" s="4" t="inlineStr">
@@ -13423,7 +13442,7 @@
       </c>
       <c r="X51" s="4" t="inlineStr">
         <is>
-          <t>5000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Y51" s="4" t="inlineStr">
@@ -13443,7 +13462,7 @@
       </c>
       <c r="AB51" s="4" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>OUTROS</t>
         </is>
       </c>
       <c r="AC51" s="4" t="inlineStr">
@@ -13493,12 +13512,12 @@
       </c>
       <c r="AL51" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["Private"]</t>
         </is>
       </c>
       <c r="AM51" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["Private"]</t>
         </is>
       </c>
       <c r="AN51" s="4" t="inlineStr">
@@ -13519,51 +13538,52 @@
       </c>
       <c r="AR51" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS51" s="4" t="inlineStr"/>
+          <t>CAIXA SIGMA PRIVATE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REF DI LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS51" s="4" t="inlineStr">
+        <is>
+          <t>A movimentação do fundo é feita exclusivamente pela plataforma.caixa ou IBC/APP.
+Fundo teve alteração de nomenclatura a partir de 21/09/2026 de CAIXA ÔMEGA PRIVATE para CAIXA SIGMA PRIVATE.</t>
+        </is>
+      </c>
       <c r="AT51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5171.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7914.pdf</t>
         </is>
       </c>
       <c r="AU51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5171.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7914.pdf</t>
         </is>
       </c>
       <c r="AV51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5171.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7914.pdf</t>
         </is>
       </c>
       <c r="AW51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7914.pdf</t>
         </is>
       </c>
       <c r="AX51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7914.pdf</t>
         </is>
       </c>
       <c r="AY51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7914.pdf</t>
         </is>
       </c>
       <c r="AZ51" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5171.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7914.pdf</t>
         </is>
       </c>
       <c r="BA51" s="4" t="inlineStr"/>
-      <c r="BB51" s="4" t="inlineStr">
-        <is>
-          <t>https://web.microsoftstream.com/video/4be15710-4acb-4afd-a959-c6ed0d090cac?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
-        </is>
-      </c>
+      <c r="BB51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14044,10 +14064,14 @@
       </c>
       <c r="AR53" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS53" s="4" t="inlineStr"/>
+          <t>CAIXA SIGMA SINGULAR FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REF DI LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS53" s="4" t="inlineStr">
+        <is>
+          <t>Fundo teve alteração de nomenclatura a partir de 21/09/2026 de CAIXA SIGMA para CAIXA SIGMA SINGULAR</t>
+        </is>
+      </c>
       <c r="AT53" s="4" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5171.pdf</t>
@@ -14690,7 +14714,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="P56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/voce/renda-fixa/caixa-turquesa-pj/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="2" t="inlineStr"/>
       <c r="S56" s="2" t="inlineStr"/>
@@ -16088,7 +16116,7 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-short-mm</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-short-mm/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
@@ -16344,7 +16372,7 @@
       </c>
       <c r="P63" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-long-bias-mm</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q63" s="4" t="inlineStr">
@@ -16852,7 +16880,7 @@
       </c>
       <c r="P65" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q65" s="4" t="inlineStr">
@@ -19440,19 +19468,15 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
-        </is>
-      </c>
+      <c r="P75" s="4" t="inlineStr"/>
       <c r="Q75" s="4" t="inlineStr">
         <is>
-          <t>34.660.333/0001-69</t>
+          <t>35.536.472/0001-48</t>
         </is>
       </c>
       <c r="R75" s="4" t="inlineStr">
         <is>
-          <t>6440</t>
+          <t>6479</t>
         </is>
       </c>
       <c r="S75" s="4" t="inlineStr">
@@ -19462,7 +19486,7 @@
       </c>
       <c r="T75" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="U75" s="4" t="inlineStr">
@@ -19550,16 +19574,8 @@
           <t>100.0</t>
         </is>
       </c>
-      <c r="AL75" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "Private"]</t>
-        </is>
-      </c>
-      <c r="AM75" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "Private"]</t>
-        </is>
-      </c>
+      <c r="AL75" s="4" t="inlineStr"/>
+      <c r="AM75" s="4" t="inlineStr"/>
       <c r="AN75" s="4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -19578,43 +19594,47 @@
       </c>
       <c r="AR75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITA</t>
-        </is>
-      </c>
-      <c r="AS75" s="4" t="inlineStr"/>
+          <t>CAIXA FUNCIONÁRIOS ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABI</t>
+        </is>
+      </c>
+      <c r="AS75" s="4" t="inlineStr">
+        <is>
+          <t>Fundo destinado a Funcionários e aposentados da Caixa Econômica Federal. Disponível para aplicação somente via conta corrente marcada como conta-salário empregado CAIXA.</t>
+        </is>
+      </c>
       <c r="AT75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6440.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6479.pdf</t>
         </is>
       </c>
       <c r="AU75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6440.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6479.pdf</t>
         </is>
       </c>
       <c r="AV75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6440.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6479.pdf</t>
         </is>
       </c>
       <c r="AW75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6440.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6479.pdf</t>
         </is>
       </c>
       <c r="AX75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6440.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6479.pdf</t>
         </is>
       </c>
       <c r="AY75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6440.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6479.pdf</t>
         </is>
       </c>
       <c r="AZ75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6440.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6479.pdf</t>
         </is>
       </c>
       <c r="BA75" s="4" t="inlineStr"/>
@@ -20481,7 +20501,7 @@
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q79" s="4" t="inlineStr">
@@ -20606,7 +20626,7 @@
       </c>
       <c r="AO79" s="4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="AP79" s="4" t="inlineStr">
@@ -22840,7 +22860,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fic-fif-quantitativo-low-vol/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q88" s="2" t="inlineStr"/>
       <c r="R88" s="2" t="inlineStr"/>
       <c r="S88" s="2" t="inlineStr"/>
@@ -22958,7 +22982,7 @@
       </c>
       <c r="P89" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fic-fia-compromisso-bdr-nivel-i</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIA-Institucional-BDR-nivel-I/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q89" s="4" t="inlineStr">
@@ -23214,7 +23238,7 @@
       </c>
       <c r="P90" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-ibovespa</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-etf-bovespa/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q90" s="2" t="inlineStr">
@@ -26587,7 +26611,7 @@
       </c>
       <c r="P103" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/Caixa-FI-Acoes-Banco-do-Brasil-Plus/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/Caixa-FI-Acoes-Banco-do-Brasil-Plus/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q103" s="4" t="inlineStr">
@@ -28913,7 +28937,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="P112" s="2" t="inlineStr"/>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-seguridade/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q112" s="2" t="inlineStr">
         <is>
           <t>59.815.671/0001-53</t>
@@ -31481,17 +31509,17 @@
       </c>
       <c r="P122" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="Q122" s="2" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="R122" s="2" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="S122" s="2" t="inlineStr">
@@ -31501,12 +31529,12 @@
       </c>
       <c r="T122" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="U122" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V122" s="2" t="inlineStr">
@@ -31601,7 +31629,7 @@
       </c>
       <c r="AR122" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS122" s="2" t="inlineStr">
@@ -31611,37 +31639,37 @@
       </c>
       <c r="AT122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
         </is>
       </c>
       <c r="AU122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="AV122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="AW122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="AX122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="AY122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="AZ122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
         </is>
       </c>
       <c r="BA122" s="2" t="inlineStr"/>
@@ -32476,17 +32504,17 @@
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="R126" s="2" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="S126" s="2" t="inlineStr">
@@ -32496,12 +32524,12 @@
       </c>
       <c r="T126" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="U126" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V126" s="2" t="inlineStr">
@@ -32596,7 +32624,7 @@
       </c>
       <c r="AR126" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS126" s="2" t="inlineStr">
@@ -32606,37 +32634,37 @@
       </c>
       <c r="AT126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
         </is>
       </c>
       <c r="AU126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="AV126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="AW126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="AX126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="AY126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="AZ126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
         </is>
       </c>
       <c r="BA126" s="2" t="inlineStr"/>
@@ -32966,7 +32994,11 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="P128" s="2" t="inlineStr"/>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>http://site.extra.caixa.gov.br/fundos-investimento/fundo-simples/fic-azulzinha-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q128" s="2" t="inlineStr">
         <is>
           <t>61.160.298/0001-91</t>
@@ -33225,7 +33257,7 @@
       </c>
       <c r="P129" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-ametista-corporativo-rf-simples</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-ametista-pj/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q129" s="4" t="inlineStr">
@@ -33631,8 +33663,7 @@
       </c>
       <c r="AS130" s="2" t="inlineStr">
         <is>
-          <t>*Nome alterado de CAIXA FIC FORTALECER RF LONGO PRAZO para CAIXA FIC EQUILIBRIO MPE RF LONGO PRAZO, em 15 JAN 2024, conforme aprovado em Assembleia Geral de Cotistas.
-Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
         </is>
       </c>
       <c r="AT130" s="2" t="inlineStr">
@@ -34574,7 +34605,7 @@
       </c>
       <c r="X134" s="2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y134" s="2" t="inlineStr">
@@ -35315,7 +35346,7 @@
       </c>
       <c r="P137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-institucional-soberano-plus-rf-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-institucional-soberano-plus-rf-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q137" s="4" t="inlineStr">
@@ -36306,7 +36337,11 @@
           <t>PJ | RPPS</t>
         </is>
       </c>
-      <c r="P141" s="4" t="inlineStr"/>
+      <c r="P141" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/referenciados/caixa-brasil-esmeralda-rf-ref/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q141" s="4" t="inlineStr">
         <is>
           <t>68.375.792/0001-12</t>
@@ -36600,7 +36635,7 @@
       </c>
       <c r="X142" s="2" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y142" s="2" t="inlineStr">
@@ -36846,7 +36881,7 @@
       </c>
       <c r="U143" s="4" t="inlineStr">
         <is>
-          <t>3000000.0</t>
+          <t>1000000.0</t>
         </is>
       </c>
       <c r="V143" s="4" t="inlineStr">
@@ -36861,7 +36896,7 @@
       </c>
       <c r="X143" s="4" t="inlineStr">
         <is>
-          <t>300000.0</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="Y143" s="4" t="inlineStr">
@@ -36960,7 +36995,15 @@
           <t>CAIXA TOPÁZIO CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
-      <c r="AS143" s="4" t="inlineStr"/>
+      <c r="AS143" s="4" t="inlineStr">
+        <is>
+          <t>Fundo em Campanha - Período 21/09/2026 à 30/12/2026
+Redução de Ticket
+Aplicação Inicial: De R$ 3.000.000,00 Para R$ 1.000.000,00
+Saldo Mínimo: De R$ 300.000,00 Para R$ 100.000,00
+"Fundos de Investimento que estiveram em Campanha, após a Campanha, voltam aos parâmetros originais. Saldo abaixo do mínimo pode impedir resgates parciais (somente total)."</t>
+        </is>
+      </c>
       <c r="AT143" s="4" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5189.pdf</t>
@@ -37447,12 +37490,12 @@
       </c>
       <c r="AL145" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
         </is>
       </c>
       <c r="AM145" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
         </is>
       </c>
       <c r="AN145" s="4" t="inlineStr">
@@ -37597,7 +37640,7 @@
       </c>
       <c r="P146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q146" s="2" t="inlineStr">
@@ -38381,12 +38424,12 @@
       </c>
       <c r="Q149" s="4" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="R149" s="4" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="S149" s="4" t="inlineStr">
@@ -38436,7 +38479,7 @@
       </c>
       <c r="AB149" s="4" t="inlineStr">
         <is>
-          <t>IRF-M TOTAL</t>
+          <t>IRF-M 1</t>
         </is>
       </c>
       <c r="AC149" s="4" t="inlineStr">
@@ -38461,17 +38504,17 @@
       </c>
       <c r="AG149" s="4" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="AH149" s="4" t="inlineStr">
         <is>
-          <t>16h00</t>
+          <t>17h00</t>
         </is>
       </c>
       <c r="AI149" s="4" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 90%</t>
+          <t>Sim · Automatico · 95%</t>
         </is>
       </c>
       <c r="AJ149" s="4" t="inlineStr">
@@ -38481,7 +38524,7 @@
       </c>
       <c r="AK149" s="4" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AL149" s="4" t="inlineStr">
@@ -38512,54 +38555,58 @@
       </c>
       <c r="AR149" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS149" s="4" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
+2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="AU149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="AV149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="AW149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="AX149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="AY149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
       <c r="AZ149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
         </is>
       </c>
       <c r="BA149" s="4" t="inlineStr"/>
-      <c r="BB149" s="4" t="inlineStr"/>
+      <c r="BB149" s="4" t="inlineStr">
+        <is>
+          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -38644,12 +38691,12 @@
       </c>
       <c r="Q150" s="2" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="R150" s="2" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="S150" s="2" t="inlineStr">
@@ -38699,7 +38746,7 @@
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
-          <t>IRF-M TOTAL</t>
+          <t>IRF-M 1</t>
         </is>
       </c>
       <c r="AC150" s="2" t="inlineStr">
@@ -38724,17 +38771,17 @@
       </c>
       <c r="AG150" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="AH150" s="2" t="inlineStr">
         <is>
-          <t>16h00</t>
+          <t>17h00</t>
         </is>
       </c>
       <c r="AI150" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 90%</t>
+          <t>Sim · Automatico · 95%</t>
         </is>
       </c>
       <c r="AJ150" s="2" t="inlineStr">
@@ -38744,7 +38791,7 @@
       </c>
       <c r="AK150" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AL150" s="2" t="inlineStr">
@@ -38775,54 +38822,58 @@
       </c>
       <c r="AR150" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS150" s="2" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
+2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="AU150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="AV150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="AW150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="AX150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="AY150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
       <c r="AZ150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
         </is>
       </c>
       <c r="BA150" s="2" t="inlineStr"/>
-      <c r="BB150" s="2" t="inlineStr"/>
+      <c r="BB150" s="2" t="inlineStr">
+        <is>
+          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -39423,7 +39474,7 @@
       </c>
       <c r="P153" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-brasil-renda-fixa-ativa-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-IPCA/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q153" s="4" t="inlineStr">
@@ -39951,12 +40002,12 @@
       </c>
       <c r="Q155" s="4" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R155" s="4" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S155" s="4" t="inlineStr">
@@ -40006,7 +40057,7 @@
       </c>
       <c r="AB155" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC155" s="4" t="inlineStr">
@@ -40082,49 +40133,43 @@
       </c>
       <c r="AR155" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS155" s="4" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS155" s="4" t="inlineStr"/>
       <c r="AT155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA155" s="4" t="inlineStr"/>
@@ -40213,12 +40258,12 @@
       </c>
       <c r="Q156" s="2" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R156" s="2" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S156" s="2" t="inlineStr">
@@ -40268,7 +40313,7 @@
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC156" s="2" t="inlineStr">
@@ -40344,49 +40389,43 @@
       </c>
       <c r="AR156" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS156" s="2" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS156" s="2" t="inlineStr"/>
       <c r="AT156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA156" s="2" t="inlineStr"/>
@@ -40857,12 +40896,12 @@
       </c>
       <c r="Q159" s="4" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R159" s="4" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S159" s="4" t="inlineStr">
@@ -40912,7 +40951,7 @@
       </c>
       <c r="AB159" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC159" s="4" t="inlineStr">
@@ -40988,49 +41027,43 @@
       </c>
       <c r="AR159" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS159" s="4" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS159" s="4" t="inlineStr"/>
       <c r="AT159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA159" s="4" t="inlineStr"/>
@@ -41119,12 +41152,12 @@
       </c>
       <c r="Q160" s="2" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="R160" s="2" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="S160" s="2" t="inlineStr">
@@ -41174,7 +41207,7 @@
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
-          <t>IRF-M TOTAL</t>
+          <t>IRF-M 1</t>
         </is>
       </c>
       <c r="AC160" s="2" t="inlineStr">
@@ -41199,17 +41232,17 @@
       </c>
       <c r="AG160" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="AH160" s="2" t="inlineStr">
         <is>
-          <t>16h00</t>
+          <t>17h00</t>
         </is>
       </c>
       <c r="AI160" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 90%</t>
+          <t>Sim · Automatico · 95%</t>
         </is>
       </c>
       <c r="AJ160" s="2" t="inlineStr">
@@ -41219,7 +41252,7 @@
       </c>
       <c r="AK160" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AL160" s="2" t="inlineStr">
@@ -41250,54 +41283,58 @@
       </c>
       <c r="AR160" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS160" s="2" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
+2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="AU160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="AV160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="AW160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="AX160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="AY160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
       <c r="AZ160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
         </is>
       </c>
       <c r="BA160" s="2" t="inlineStr"/>
-      <c r="BB160" s="2" t="inlineStr"/>
+      <c r="BB160" s="2" t="inlineStr">
+        <is>
+          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -41377,7 +41414,7 @@
       </c>
       <c r="P161" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-matriz-rf/</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-matriz-rf/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q161" s="4" t="inlineStr">
@@ -41646,12 +41683,12 @@
       </c>
       <c r="Q162" s="2" t="inlineStr">
         <is>
-          <t>03.737.206/0001-97</t>
+          <t>05.164.356/0001-84</t>
         </is>
       </c>
       <c r="R162" s="2" t="inlineStr">
         <is>
-          <t>5404</t>
+          <t>5462</t>
         </is>
       </c>
       <c r="S162" s="2" t="inlineStr">
@@ -41706,7 +41743,7 @@
       </c>
       <c r="AC162" s="2" t="inlineStr">
         <is>
-          <t>RF DI até 49% Crédito Privado</t>
+          <t>RF 100% TPF - Longo Prazo</t>
         </is>
       </c>
       <c r="AD162" s="2" t="inlineStr">
@@ -41777,54 +41814,53 @@
       </c>
       <c r="AR162" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA BRASIL TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS162" s="2" t="inlineStr">
         <is>
-          <t>1. Para aplicação por meio de conta operação 003, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-2. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 003, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
+          <t>Para aplicação no fundo é necessário o cadastramento prévio de cotistas, conforme descrito no FI657. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação, mesmo para os clientes que já realizaram o cadsatramento anteriormente.</t>
         </is>
       </c>
       <c r="AT162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
         </is>
       </c>
       <c r="AU162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
         </is>
       </c>
       <c r="AV162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
         </is>
       </c>
       <c r="AW162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
         </is>
       </c>
       <c r="AX162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
         </is>
       </c>
       <c r="AY162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
         </is>
       </c>
       <c r="AZ162" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5462.pdf</t>
         </is>
       </c>
       <c r="BA162" s="2" t="inlineStr"/>
       <c r="BB162" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/f88f1fc7-aac3-44df-a2a5-ce3ac05edfb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -42691,7 +42727,7 @@
       </c>
       <c r="S166" s="2" t="inlineStr">
         <is>
-          <t>Conservador</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="T166" s="2" t="inlineStr">
@@ -42947,7 +42983,7 @@
       </c>
       <c r="S167" s="4" t="inlineStr">
         <is>
-          <t>Conservador</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="T167" s="4" t="inlineStr">
@@ -43203,7 +43239,7 @@
       </c>
       <c r="S168" s="2" t="inlineStr">
         <is>
-          <t>Conservador</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="T168" s="2" t="inlineStr">
@@ -43548,8 +43584,16 @@
         </is>
       </c>
       <c r="AK169" s="4" t="inlineStr"/>
-      <c r="AL169" s="4" t="inlineStr"/>
-      <c r="AM169" s="4" t="inlineStr"/>
+      <c r="AL169" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AM169" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "RPPS"]</t>
+        </is>
+      </c>
       <c r="AN169" s="4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -43707,7 +43751,7 @@
       </c>
       <c r="S170" s="2" t="inlineStr">
         <is>
-          <t>Conservador</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="T170" s="2" t="inlineStr">
@@ -43963,7 +44007,7 @@
       </c>
       <c r="S171" s="4" t="inlineStr">
         <is>
-          <t>Conservador</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="T171" s="4" t="inlineStr">
@@ -44589,7 +44633,7 @@
       </c>
       <c r="P174" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/rpps/brasil-estrategia-livre-mm-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q174" s="2" t="inlineStr">
@@ -44846,12 +44890,12 @@
       </c>
       <c r="Q175" s="4" t="inlineStr">
         <is>
-          <t>15.154.236/0001-50</t>
+          <t>13.058.816/0001-18</t>
         </is>
       </c>
       <c r="R175" s="4" t="inlineStr">
         <is>
-          <t>5842</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="S175" s="4" t="inlineStr">
@@ -44911,7 +44955,7 @@
       </c>
       <c r="AD175" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE175" s="4" t="inlineStr">
@@ -44977,47 +45021,43 @@
       </c>
       <c r="AR175" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL ETF IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS175" s="4" t="inlineStr">
-        <is>
-          <t>Fundo fechado para novas aplicações, a novos investidores e cotistas atuais a partir de 03/04/2023 (inclusive)</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL INDEXA IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS175" s="4" t="inlineStr"/>
       <c r="AT175" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5445.pdf</t>
         </is>
       </c>
       <c r="AU175" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5445.pdf</t>
         </is>
       </c>
       <c r="AV175" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5445.pdf</t>
         </is>
       </c>
       <c r="AW175" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5445.pdf</t>
         </is>
       </c>
       <c r="AX175" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
         </is>
       </c>
       <c r="AY175" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
         </is>
       </c>
       <c r="AZ175" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5445.pdf</t>
         </is>
       </c>
       <c r="BA175" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 28/10/2026 16:04
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -2178,12 +2178,12 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>40.194.314/0001-97</t>
+          <t>40.194.309/0001-84</t>
         </is>
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>6532</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
@@ -2193,27 +2193,27 @@
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V7" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="X7" s="4" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y7" s="4" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="AF7" s="4" t="inlineStr">
         <is>
-          <t>QUALIFICADO</t>
+          <t>GERAL</t>
         </is>
       </c>
       <c r="AG7" s="4" t="inlineStr">
@@ -2309,47 +2309,43 @@
       </c>
       <c r="AR7" s="4" t="inlineStr">
         <is>
-          <t>CAIXA PLUS QUALIFICADO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LP - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS7" s="4" t="inlineStr">
-        <is>
-          <t>OBS: Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
-        </is>
-      </c>
+          <t>CAIXA PLUS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS7" s="4" t="inlineStr"/>
       <c r="AT7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6533.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6532.pdf</t>
         </is>
       </c>
       <c r="AU7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6533.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6532.pdf</t>
         </is>
       </c>
       <c r="AV7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6533.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6532.pdf</t>
         </is>
       </c>
       <c r="AW7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6533.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6532.pdf</t>
         </is>
       </c>
       <c r="AX7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6533.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6532.pdf</t>
         </is>
       </c>
       <c r="AY7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6533.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6532.pdf</t>
         </is>
       </c>
       <c r="AZ7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6533.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6532.pdf</t>
         </is>
       </c>
       <c r="BA7" s="4" t="inlineStr"/>
@@ -2632,7 +2628,11 @@
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AG9" s="4" t="inlineStr"/>
+      <c r="AG9" s="4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
       <c r="AH9" s="4" t="inlineStr">
         <is>
           <t>17h00</t>
@@ -3178,12 +3178,12 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>03.218.183/0001-04</t>
+          <t>03.191.874/0001-61</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>46</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -3193,27 +3193,27 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -3283,12 +3283,12 @@
       </c>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
@@ -3319,43 +3319,43 @@
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
         </is>
       </c>
       <c r="AX12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
       <c r="AY12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
         </is>
       </c>
       <c r="AZ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
         </is>
       </c>
       <c r="BA12" s="2" t="inlineStr"/>
       <c r="BB12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/32d65536-1de1-4f2f-a9b8-0fbb0d9347fc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="U45" s="4" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>50000.0</t>
         </is>
       </c>
       <c r="V45" s="4" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="X45" s="4" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>5000.0</t>
         </is>
       </c>
       <c r="Y45" s="4" t="inlineStr">
@@ -11839,7 +11839,14 @@
       </c>
       <c r="AS45" s="4" t="inlineStr">
         <is>
-          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).
+Campanha "Semana do Consumidor" de 26/10/2026 a 30/10/2026
+Redução de Tickets
+Aplicação Inicial:
+De: R$ 100.000,00 para R$ 50.000,00
+Saldo Mínimo: 
+De: R$ 10.000,00 para R$ 5.000,00
+"Fundos de Investimento que estiveram em Campanha, após a Campanha, voltam aos parâmetros originais. Saldo abaixo do mínimo pode impedir resgates parciais (somente total)."</t>
         </is>
       </c>
       <c r="AT45" s="4" t="inlineStr">
@@ -12220,19 +12227,15 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P47" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/referenciados/fic-sigma-ref-di-longo-prazo</t>
-        </is>
-      </c>
+      <c r="P47" s="4" t="inlineStr"/>
       <c r="Q47" s="4" t="inlineStr">
         <is>
-          <t>10.731.794/0001-17</t>
+          <t>69.516.203/0001-31</t>
         </is>
       </c>
       <c r="R47" s="4" t="inlineStr">
         <is>
-          <t>5171</t>
+          <t>7989</t>
         </is>
       </c>
       <c r="S47" s="4" t="inlineStr">
@@ -12242,27 +12245,27 @@
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="U47" s="4" t="inlineStr">
         <is>
-          <t>50000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V47" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="X47" s="4" t="inlineStr">
         <is>
-          <t>5000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y47" s="4" t="inlineStr">
@@ -12332,12 +12335,12 @@
       </c>
       <c r="AL47" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["Pessoa Física", "Private"]</t>
         </is>
       </c>
       <c r="AM47" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["Pessoa Física", "Private"]</t>
         </is>
       </c>
       <c r="AN47" s="4" t="inlineStr">
@@ -12358,55 +12361,47 @@
       </c>
       <c r="AR47" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA SINGULAR FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REF DI LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS47" s="4" t="inlineStr">
-        <is>
-          <t>Fundo teve alteração de nomenclatura a partir de 21/09/2026 de CAIXA SIGMA para CAIXA SIGMA SINGULAR</t>
-        </is>
-      </c>
+          <t>CAIXA SIGMA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS47" s="4" t="inlineStr"/>
       <c r="AT47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5171.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7989.pdf</t>
         </is>
       </c>
       <c r="AU47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5171.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7989.pdf</t>
         </is>
       </c>
       <c r="AV47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7989.pdf</t>
         </is>
       </c>
       <c r="AW47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7989.pdf</t>
         </is>
       </c>
       <c r="AX47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7989.pdf</t>
         </is>
       </c>
       <c r="AY47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7989.pdf</t>
         </is>
       </c>
       <c r="AZ47" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5171.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7989.pdf</t>
         </is>
       </c>
       <c r="BA47" s="4" t="inlineStr"/>
-      <c r="BB47" s="4" t="inlineStr">
-        <is>
-          <t>https://web.microsoftstream.com/video/4be15710-4acb-4afd-a959-c6ed0d090cac?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
-        </is>
-      </c>
+      <c r="BB47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14601,7 +14596,7 @@
       </c>
       <c r="U56" s="2" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>50000.0</t>
         </is>
       </c>
       <c r="V56" s="2" t="inlineStr">
@@ -14616,7 +14611,7 @@
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>5000.0</t>
         </is>
       </c>
       <c r="Y56" s="2" t="inlineStr">
@@ -14715,7 +14710,17 @@
           <t>CAIXA MEGA FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
-      <c r="AS56" s="2" t="inlineStr"/>
+      <c r="AS56" s="2" t="inlineStr">
+        <is>
+          <t>Campanha "Semana do Consumidor" de 26/10/2026 a 30/10/2026
+Redução de Tickets
+Aplicação Inicial:
+De: R$ 100.000,00 para R$ 50.000,00
+Saldo Mínimo: 
+De: R$ 10.000,00 para R$ 5.000,00
+"Fundos de Investimento que estiveram em Campanha, após a Campanha, voltam aos parâmetros originais. Saldo abaixo do mínimo pode impedir resgates parciais (somente total)."</t>
+        </is>
+      </c>
       <c r="AT56" s="2" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5411.pdf</t>
@@ -15098,43 +15103,187 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="P58" s="2" t="inlineStr"/>
-      <c r="Q58" s="2" t="inlineStr"/>
-      <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="2" t="inlineStr"/>
-      <c r="T58" s="2" t="inlineStr"/>
-      <c r="U58" s="2" t="inlineStr"/>
-      <c r="V58" s="2" t="inlineStr"/>
-      <c r="W58" s="2" t="inlineStr"/>
-      <c r="X58" s="2" t="inlineStr"/>
-      <c r="Y58" s="2" t="inlineStr"/>
-      <c r="Z58" s="2" t="inlineStr"/>
-      <c r="AA58" s="2" t="inlineStr"/>
-      <c r="AB58" s="2" t="inlineStr"/>
-      <c r="AC58" s="2" t="inlineStr"/>
-      <c r="AD58" s="2" t="inlineStr"/>
-      <c r="AE58" s="2" t="inlineStr"/>
-      <c r="AF58" s="2" t="inlineStr"/>
-      <c r="AG58" s="2" t="inlineStr"/>
-      <c r="AH58" s="2" t="inlineStr"/>
-      <c r="AI58" s="2" t="inlineStr"/>
-      <c r="AJ58" s="2" t="inlineStr"/>
-      <c r="AK58" s="2" t="inlineStr"/>
-      <c r="AL58" s="2" t="inlineStr"/>
-      <c r="AM58" s="2" t="inlineStr"/>
-      <c r="AN58" s="2" t="inlineStr"/>
-      <c r="AO58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/voce/renda-fixa/caixa-fic-rf-curto-prazo</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>6520</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="inlineStr">
+        <is>
+          <t>RF 100% TPF - Curto Prazo</t>
+        </is>
+      </c>
+      <c r="AD58" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE58" s="2" t="inlineStr">
+        <is>
+          <t>CURTO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF58" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AG58" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AH58" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI58" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AJ58" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK58" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AL58" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM58" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN58" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO58" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP58" s="2" t="inlineStr"/>
-      <c r="AQ58" s="2" t="inlineStr"/>
-      <c r="AR58" s="2" t="inlineStr"/>
-      <c r="AS58" s="2" t="inlineStr"/>
-      <c r="AT58" s="2" t="inlineStr"/>
-      <c r="AU58" s="2" t="inlineStr"/>
-      <c r="AV58" s="2" t="inlineStr"/>
-      <c r="AW58" s="2" t="inlineStr"/>
-      <c r="AX58" s="2" t="inlineStr"/>
-      <c r="AY58" s="2" t="inlineStr"/>
-      <c r="AZ58" s="2" t="inlineStr"/>
+      <c r="AQ58" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR58" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA TURQUESA PJ FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS58" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AT58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AU58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AV58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AW58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AX58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AY58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AZ58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
+        </is>
+      </c>
       <c r="BA58" s="2" t="inlineStr"/>
       <c r="BB58" s="2" t="inlineStr"/>
     </row>
@@ -19848,15 +19997,19 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P77" s="4" t="inlineStr"/>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q77" s="4" t="inlineStr">
         <is>
-          <t>35.536.472/0001-48</t>
+          <t>34.660.333/0001-69</t>
         </is>
       </c>
       <c r="R77" s="4" t="inlineStr">
         <is>
-          <t>6479</t>
+          <t>6440</t>
         </is>
       </c>
       <c r="S77" s="4" t="inlineStr">
@@ -19866,7 +20019,7 @@
       </c>
       <c r="T77" s="4" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U77" s="4" t="inlineStr">
@@ -19954,8 +20107,16 @@
           <t>100.0</t>
         </is>
       </c>
-      <c r="AL77" s="4" t="inlineStr"/>
-      <c r="AM77" s="4" t="inlineStr"/>
+      <c r="AL77" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM77" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
       <c r="AN77" s="4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -19974,47 +20135,43 @@
       </c>
       <c r="AR77" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FUNCIONÁRIOS ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABI</t>
-        </is>
-      </c>
-      <c r="AS77" s="4" t="inlineStr">
-        <is>
-          <t>Fundo destinado a Funcionários e aposentados da Caixa Econômica Federal. Disponível para aplicação somente via conta corrente marcada como conta-salário empregado CAIXA.</t>
-        </is>
-      </c>
+          <t>CAIXA ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITA</t>
+        </is>
+      </c>
+      <c r="AS77" s="4" t="inlineStr"/>
       <c r="AT77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6440.pdf</t>
         </is>
       </c>
       <c r="AU77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6440.pdf</t>
         </is>
       </c>
       <c r="AV77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6440.pdf</t>
         </is>
       </c>
       <c r="AW77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6440.pdf</t>
         </is>
       </c>
       <c r="AX77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6440.pdf</t>
         </is>
       </c>
       <c r="AY77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6440.pdf</t>
         </is>
       </c>
       <c r="AZ77" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6440.pdf</t>
         </is>
       </c>
       <c r="BA77" s="4" t="inlineStr"/>
@@ -31885,17 +32042,17 @@
       </c>
       <c r="P124" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="R124" s="2" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="S124" s="2" t="inlineStr">
@@ -31905,12 +32062,12 @@
       </c>
       <c r="T124" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="U124" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V124" s="2" t="inlineStr">
@@ -32005,7 +32162,7 @@
       </c>
       <c r="AR124" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS124" s="2" t="inlineStr">
@@ -32015,37 +32172,37 @@
       </c>
       <c r="AT124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
         </is>
       </c>
       <c r="AU124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="AV124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="AW124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="AX124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="AY124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="AZ124" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
         </is>
       </c>
       <c r="BA124" s="2" t="inlineStr"/>
@@ -32880,17 +33037,17 @@
       </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="R128" s="2" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="S128" s="2" t="inlineStr">
@@ -32900,12 +33057,12 @@
       </c>
       <c r="T128" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="U128" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V128" s="2" t="inlineStr">
@@ -33000,7 +33157,7 @@
       </c>
       <c r="AR128" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS128" s="2" t="inlineStr">
@@ -33010,37 +33167,37 @@
       </c>
       <c r="AT128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
         </is>
       </c>
       <c r="AU128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="AV128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="AW128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="AX128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="AY128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="AZ128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
         </is>
       </c>
       <c r="BA128" s="2" t="inlineStr"/>
@@ -40377,12 +40534,12 @@
       </c>
       <c r="Q157" s="4" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R157" s="4" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S157" s="4" t="inlineStr">
@@ -40432,7 +40589,7 @@
       </c>
       <c r="AB157" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC157" s="4" t="inlineStr">
@@ -40508,49 +40665,43 @@
       </c>
       <c r="AR157" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS157" s="4" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS157" s="4" t="inlineStr"/>
       <c r="AT157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA157" s="4" t="inlineStr"/>
@@ -40639,12 +40790,12 @@
       </c>
       <c r="Q158" s="2" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R158" s="2" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S158" s="2" t="inlineStr">
@@ -40694,7 +40845,7 @@
       </c>
       <c r="AB158" s="2" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC158" s="2" t="inlineStr">
@@ -40770,49 +40921,43 @@
       </c>
       <c r="AR158" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS158" s="2" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS158" s="2" t="inlineStr"/>
       <c r="AT158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA158" s="2" t="inlineStr"/>
@@ -41283,12 +41428,12 @@
       </c>
       <c r="Q161" s="4" t="inlineStr">
         <is>
-          <t>10.577.503/0001-88</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R161" s="4" t="inlineStr">
         <is>
-          <t>5568</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S161" s="4" t="inlineStr">
@@ -41338,7 +41483,7 @@
       </c>
       <c r="AB161" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5+</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC161" s="4" t="inlineStr">
@@ -41414,49 +41559,43 @@
       </c>
       <c r="AR161" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS161" s="4" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS161" s="4" t="inlineStr"/>
       <c r="AT161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA161" s="4" t="inlineStr"/>
@@ -45283,12 +45422,12 @@
       </c>
       <c r="Q177" s="4" t="inlineStr">
         <is>
-          <t>15.154.236/0001-50</t>
+          <t>13.058.816/0001-18</t>
         </is>
       </c>
       <c r="R177" s="4" t="inlineStr">
         <is>
-          <t>5842</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="S177" s="4" t="inlineStr">
@@ -45348,7 +45487,7 @@
       </c>
       <c r="AD177" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE177" s="4" t="inlineStr">
@@ -45414,47 +45553,43 @@
       </c>
       <c r="AR177" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL ETF IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS177" s="4" t="inlineStr">
-        <is>
-          <t>Fundo fechado para novas aplicações, a novos investidores e cotistas atuais a partir de 03/04/2023 (inclusive)</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL INDEXA IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS177" s="4" t="inlineStr"/>
       <c r="AT177" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5445.pdf</t>
         </is>
       </c>
       <c r="AU177" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5445.pdf</t>
         </is>
       </c>
       <c r="AV177" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5445.pdf</t>
         </is>
       </c>
       <c r="AW177" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5445.pdf</t>
         </is>
       </c>
       <c r="AX177" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
         </is>
       </c>
       <c r="AY177" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
         </is>
       </c>
       <c r="AZ177" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5445.pdf</t>
         </is>
       </c>
       <c r="BA177" s="4" t="inlineStr"/>

</xml_diff>